<commit_message>
add a lottt of things
</commit_message>
<xml_diff>
--- a/Scrape Logic/data_nha_rieng.xlsx
+++ b/Scrape Logic/data_nha_rieng.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\estates-scraping-final\Scrape Logic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D78CBBA-BE62-4425-A4A8-6A07EF57A1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010F84D5-73D6-4A8D-AE91-968A510099A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
   <si>
     <t>STT</t>
   </si>
@@ -344,9 +345,6 @@
 - Xe ba gác vào nhà: 3m</t>
   </si>
   <si>
-    <t>Trích xuất từ trường thông tin "Đường vào" trong bài đăng nếu giá trị đủ lớn. Nếu không có thì scrape từ miêu tả và tiêu đề của bài đăng</t>
-  </si>
-  <si>
     <t>Nếu giá trị "Đường vào" không lớn hơn 50m thì sẽ được lấy từ miêu tả và tiêu đề:
 - Nếu nhà nằm trên mặt phố thì khoảng cách = 0 
 - Nếu có thông tin cách mặt đường bao nhiêu m, bao nhiêu m ra mặt đường thì sẽ trích xuất khoảng cách từ các cụm này
@@ -358,6 +356,27 @@
   <si>
     <t xml:space="preserve">Nếu trong phần miêu tả hay tiêu đề có cụm "đất trồng" thì đất sẽ được phân vào loại hỗn hợp, còn không tất cả đều được quy về trường hợp đất ở
 </t>
+  </si>
+  <si>
+    <t>Trích xuất</t>
+  </si>
+  <si>
+    <t>Nội suy</t>
+  </si>
+  <si>
+    <t>Cách thu thập</t>
+  </si>
+  <si>
+    <t>Tất cả cùng 1 giá trị</t>
+  </si>
+  <si>
+    <t>Để trống</t>
+  </si>
+  <si>
+    <t>Trích xuất + Nội suy</t>
+  </si>
+  <si>
+    <t>Trích xuất từ trường thông tin "Đường vào" trong bài đăng nếu giá trị đủ lớn. Nếu không có thì lấy từ miêu tả và tiêu đề của bài đăng</t>
   </si>
 </sst>
 </file>
@@ -389,12 +408,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -409,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -418,14 +449,58 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -701,16 +776,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
     <col min="2" max="2" width="17.140625" style="3" customWidth="1"/>
     <col min="3" max="3" width="35.28515625" style="3" customWidth="1"/>
     <col min="4" max="4" width="66.140625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -721,10 +797,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -734,8 +813,11 @@
       <c r="C2" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -745,8 +827,11 @@
       <c r="C3" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -756,8 +841,11 @@
       <c r="C4" s="3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -770,8 +858,11 @@
       <c r="D5" s="3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -784,8 +875,11 @@
       <c r="D6" s="3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -795,8 +889,11 @@
       <c r="C7" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -806,8 +903,11 @@
       <c r="C8" s="3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -817,8 +917,11 @@
       <c r="C9" s="3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -828,8 +931,11 @@
       <c r="C10" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -839,19 +945,26 @@
       <c r="C11" s="3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="E11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="8"/>
+      <c r="E12" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -861,78 +974,96 @@
       <c r="C13" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="240.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="E14" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="240.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="8" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="E15" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="153.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="E16" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="153.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="E17" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="5" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -942,22 +1073,28 @@
       <c r="C19" s="3" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="285" x14ac:dyDescent="0.25">
-      <c r="A20">
+      <c r="E19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="285" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E20" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -967,106 +1104,130 @@
       <c r="C21" s="3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="E21" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="E22" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="7" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A24">
+      <c r="E23" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="5" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="210" x14ac:dyDescent="0.25">
-      <c r="A25">
+      <c r="E24" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="210" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="5" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="225" x14ac:dyDescent="0.25">
-      <c r="A26">
+      <c r="E25" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="225" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="5" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A27">
+      <c r="E26" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="E27" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1076,8 +1237,11 @@
       <c r="C29" s="3" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E29" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1087,8 +1251,11 @@
       <c r="C30" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="E30" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1097,6 +1264,9 @@
       </c>
       <c r="C31" s="3" t="s">
         <v>64</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>